<commit_message>
Basic reqd write of excel
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python Practice\Git_Demo\openpyxl-program\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15CAC750-71E7-415C-8B69-43B257E64520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB0F28B9-77B4-4150-8059-916EC33B437E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -474,6 +474,9 @@
       <c r="C2">
         <v>1234</v>
       </c>
+      <c r="D2">
+        <v>1.256</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">

</xml_diff>